<commit_message>
Refactor: Implementacion de Web App Flask con Playwright y Dockerfile multistage para Caso 2
</commit_message>
<xml_diff>
--- a/resultado_consulta.xlsx
+++ b/resultado_consulta.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resultados'!$A$1:$J$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +27,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B4F71"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +57,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,118 +430,127 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="39" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>dni</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>miembro_de_mesa</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>nombres</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ubicación</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>dirección</t>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DNI</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Estado / cargo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nombres y apellidos</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Región / Provincia / Distrito</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Local de votación</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Referencia</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>N° de mesa</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>N° de orden</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Observación</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>10526358</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>No disponible / No disponible / No disponible</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>15121313</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>No disponible / No disponible / No disponible</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>60069778</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>No disponible / No disponible / No disponible</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>No disponible</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>61009768</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NO ERES MIEMBRO DE MESA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CALEP OMAR NEYRA TAYPE</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>LIMA / LIMA / VILLA EL SALVADOR</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>IE 7097 VILLA AMSTELVEEN</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>SECTOR 3 GRUPO 8 MZ J1 LT 4</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>CRUCE AV 3 DE OCTUBRE Y AV REVOLUCION</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>059952</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Consulta correcta</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>